<commit_message>
verification(rs2): vp077a gets its seepage mesh back; rj020 gets a circle that closes
The RS2-40-seep-d30 row had no stem of its own, so its figure run wrote
the 4,656-node FEM mesh over vp077a_mesh.json, the 2,586-node mesh that
vp077a_seep.csv is indexed on (bf76da80). The mesh is restored from before
that commit and passes u = gamma_w (h - y) at every saturated node; the d30
results keep their content under their own stem, and the figure script
now refuses to write a mesh over one a shipped seepage field is indexed on.

rj020's toe circle (R = 120 m) left the section before returning to the
ground, so its first circle could not be sliced. The builder now places it
through a face point and a crest point; only the first circle changed, and
the joints group reproduces 23/23.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XjjT2aBxw8gY7EFdpoUcpj
</commit_message>
<xml_diff>
--- a/docs/verification/files/rocscience/joints/rj020.xlsx
+++ b/docs/verification/files/rocscience/joints/rj020.xlsx
@@ -58833,10 +58833,10 @@
         <v>1</v>
       </c>
       <c r="B3" s="3">
-        <v>20.0</v>
+        <v>-1.5625</v>
       </c>
       <c r="C3" s="3">
-        <v>130.0</v>
+        <v>80.0</v>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
@@ -58844,7 +58844,7 @@
         </is>
       </c>
       <c r="E3" s="3">
-        <v>9.5840542121</v>
+        <v>22.5603237627</v>
       </c>
       <c r="F3" s="3"/>
       <c r="G3" s="3"/>

</xml_diff>